<commit_message>
Update: all changes to app, admin, utils, and output files
</commit_message>
<xml_diff>
--- a/template/template_cv.xlsx
+++ b/template/template_cv.xlsx
@@ -7,25 +7,28 @@
   </sheets>
   <definedNames>
     <definedName name="RIBA_AYU_WULANDARI">"RIBA AYU WULANDARI"</definedName>
+    <definedName name="Excel_BuiltIn_Print_Area">#REF!</definedName>
     <definedName localSheetId="0" name="Excel_BuiltIn_Print_Area">#REF!</definedName>
-    <definedName name="Excel_BuiltIn_Print_Area">#REF!</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="gU6N8uwJoRvjILcYYFlNs0Sc8/0sceCddJVdCgbXviY="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="IXGDg60FmAstesh3fnqC3GsO+Kh9i3Dpj9YY4ReoxKY="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="57">
   <si>
     <t xml:space="preserve">No. </t>
   </si>
   <si>
-    <t>2026年5月10日</t>
+    <t>LPK MIRAI CROWN INDONESIA</t>
+  </si>
+  <si>
+    <t>2026年5月15日</t>
   </si>
   <si>
     <t>姓名
@@ -36,28 +39,19 @@
 Furigana</t>
   </si>
   <si>
-    <t>マウルアナ・アイ</t>
+    <t>-</t>
   </si>
   <si>
     <t>英字表記
 Alphabet</t>
   </si>
   <si>
-    <t>maulana abdi</t>
-  </si>
-  <si>
     <t>現住所
 Kode Pos dan Alamat</t>
   </si>
   <si>
-    <t>, , , ,  - , , Indonesia</t>
-  </si>
-  <si>
     <t>生年月日
 Tanggal Lahir</t>
-  </si>
-  <si>
-    <t>2000年1月1日</t>
   </si>
   <si>
     <t>年齢
@@ -71,21 +65,12 @@
 JK</t>
   </si>
   <si>
-    <t>男            Pria</t>
-  </si>
-  <si>
     <t>電話番号
 No Handphone</t>
   </si>
   <si>
-    <t>+62</t>
-  </si>
-  <si>
     <t>宗教
 Agama</t>
-  </si>
-  <si>
-    <t>イスラム教　   Islam</t>
   </si>
   <si>
     <t>身長
@@ -99,21 +84,12 @@
 Golongan Darah</t>
   </si>
   <si>
-    <t>A型</t>
-  </si>
-  <si>
     <t>婚姻
 Status</t>
   </si>
   <si>
-    <t>未婚 Single</t>
-  </si>
-  <si>
     <t>子供
 Anak</t>
-  </si>
-  <si>
-    <t>無 　Tidak</t>
   </si>
   <si>
     <t>体重
@@ -125,9 +101,6 @@
   <si>
     <t>パスポート
 Paspor</t>
-  </si>
-  <si>
-    <t>有      Ada</t>
   </si>
   <si>
     <t>学歴
@@ -173,18 +146,18 @@
 Posisi</t>
   </si>
   <si>
-    <t>2020年</t>
-  </si>
-  <si>
-    <t>4月</t>
-  </si>
-  <si>
     <t>外国語
 Bahasa Asing</t>
   </si>
   <si>
+    <t>日本語学習期間</t>
+  </si>
+  <si>
     <t>訪日経験
 Pernah ke Jepang</t>
+  </si>
+  <si>
+    <t>--</t>
   </si>
   <si>
     <t>渡航経験
@@ -205,19 +178,25 @@
     <t>緊急連絡先</t>
   </si>
   <si>
+    <t>名</t>
+  </si>
+  <si>
+    <t>連絡先</t>
+  </si>
+  <si>
+    <t>Kontak darurat</t>
+  </si>
+  <si>
     <t>Nama</t>
   </si>
   <si>
     <t>Nomor kontak</t>
   </si>
   <si>
-    <t>Kontak darurat</t>
+    <t>目的</t>
   </si>
   <si>
-    <t>志望理由</t>
-  </si>
-  <si>
-    <t>Alasan untuk melamar</t>
+    <t>TUJUAN</t>
   </si>
   <si>
     <t>趣味
@@ -236,20 +215,25 @@
 Kekurangan</t>
   </si>
   <si>
-    <t>その他事項</t>
+    <t>運転できる</t>
   </si>
   <si>
-    <t>ket.lain-lain</t>
+    <t>運転免許証所持</t>
+  </si>
+  <si>
+    <t>Bisa Berkendara</t>
+  </si>
+  <si>
+    <t>Sim Yang Dimiliki</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy&quot;年&quot;m&quot;月&quot;d&quot;日&quot;"/>
-    <numFmt numFmtId="165" formatCode="yyyy&quot;年&quot;m&quot;月&quot;"/>
-    <numFmt numFmtId="166" formatCode="[$IDR]\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="[$IDR]\ #,##0.00"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -278,18 +262,18 @@
     <font/>
     <font>
       <b/>
+      <sz val="13.0"/>
+      <color rgb="FFCC0000"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12.0"/>
       <color rgb="FF000000"/>
       <name val="Meiryo"/>
     </font>
     <font>
       <sz val="11.0"/>
-      <color rgb="FF000000"/>
-      <name val="Meiryo"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Meiryo"/>
     </font>
@@ -353,14 +337,10 @@
       <name val="Times New Roman"/>
     </font>
     <font>
-      <sz val="13.0"/>
-      <color rgb="FF000000"/>
+      <b/>
+      <sz val="8.0"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
-    </font>
-    <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
-      <name val="Meiryo"/>
     </font>
     <font>
       <b/>
@@ -373,8 +353,14 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -387,8 +373,20 @@
         <bgColor rgb="FFBDD6EE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD6ED"/>
+        <bgColor rgb="FFBDD6ED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="51">
+  <borders count="47">
     <border/>
     <border>
       <left style="medium">
@@ -399,6 +397,22 @@
       </top>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top style="medium">
         <color rgb="FF000000"/>
       </top>
@@ -415,25 +429,7 @@
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <bottom style="medium">
+      <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
     </border>
@@ -441,17 +437,11 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
     </border>
     <border>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -460,9 +450,14 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top style="thin">
+      <bottom style="thin">
         <color rgb="FF000000"/>
-      </top>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -509,20 +504,42 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-    </border>
-    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -544,27 +561,6 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -614,14 +610,6 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -679,6 +667,11 @@
       </bottom>
     </border>
     <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+    </border>
+    <border>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -708,14 +701,6 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
     </border>
     <border>
       <left style="medium">
@@ -760,31 +745,11 @@
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <top/>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
     </border>
     <border>
-      <top/>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
@@ -793,7 +758,6 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top/>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
@@ -806,11 +770,19 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
+    <border>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="97">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -822,24 +794,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="5" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="3" fillId="0" fontId="5" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="2" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
+    <xf borderId="8" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="9" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="10" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="11" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="1" vertical="center" wrapText="0"/>
     </xf>
@@ -849,187 +822,200 @@
     <xf borderId="13" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="14" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="12" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="15" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="16" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="15" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="16" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="17" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="18" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="19" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="19" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="20" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="21" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="16" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="19" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="21" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="20" fillId="0" fontId="14" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="7" fillId="0" fontId="14" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="22" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="21" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="22" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="23" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="15" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="18" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="15" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="23" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="24" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="25" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="16" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="24" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="7" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="26" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="25" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="18" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="26" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf quotePrefix="1" borderId="20" fillId="0" fontId="14" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="27" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="27" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="27" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="16" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="18" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="28" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="29" fillId="2" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="30" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="31" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="32" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="33" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="18" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="29" fillId="2" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="20" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="34" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="27" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="35" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="18" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="24" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="24" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="36" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="16" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="16" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="18" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="16" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="17" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="21" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="20" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="28" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="29" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="37" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="38" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="24" fillId="3" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="30" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="24" fillId="0" fontId="14" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="30" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="39" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf borderId="40" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="41" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="3" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf borderId="37" fillId="2" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="24" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="39" fillId="2" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf borderId="29" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="29" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="29" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="30" fillId="4" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf borderId="19" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="30" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="31" fillId="2" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf borderId="20" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="32" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="33" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="34" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="42" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="18" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment vertical="center"/>
+    <xf borderId="43" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="44" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="45" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="31" fillId="2" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="35" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="36" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="10" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="32" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="37" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="22" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="25" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="38" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="0" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="19" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="19" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="39" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="40" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="25" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="32" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="25" fillId="0" fontId="14" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="25" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="32" fillId="0" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="41" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="42" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="43" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="25" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="20" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="44" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="45" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="46" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="17" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="47" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="48" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="49" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="50" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1042,15 +1028,43 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1381125" cy="1905000"/>
+    <xdr:ext cx="190500" cy="190500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr descr="Picture" id="0" name="image1.png"/>
+        <xdr:cNvPr id="0" name="image1.jpg" title="Gambar"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="190500" cy="190500"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.jpg" title="Gambar"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1275,24 +1289,25 @@
     <col customWidth="1" min="1" max="1" width="2.71"/>
     <col customWidth="1" min="2" max="2" width="5.57"/>
     <col customWidth="1" min="3" max="3" width="7.71"/>
-    <col customWidth="1" min="4" max="5" width="3.86"/>
+    <col customWidth="1" min="4" max="4" width="3.86"/>
+    <col customWidth="1" min="5" max="5" width="5.29"/>
     <col customWidth="1" min="6" max="6" width="10.86"/>
     <col customWidth="1" min="7" max="7" width="6.43"/>
     <col customWidth="1" min="8" max="8" width="5.29"/>
     <col customWidth="1" min="9" max="9" width="12.14"/>
     <col customWidth="1" min="10" max="10" width="7.29"/>
     <col customWidth="1" min="11" max="11" width="18.57"/>
-    <col customWidth="1" min="12" max="12" width="8.43"/>
-    <col customWidth="1" min="13" max="13" width="8.71"/>
-    <col customWidth="1" min="14" max="14" width="5.43"/>
-    <col customWidth="1" min="15" max="15" width="4.71"/>
-    <col customWidth="1" min="16" max="16" width="6.14"/>
-    <col customWidth="1" min="17" max="17" width="6.0"/>
-    <col customWidth="1" min="18" max="18" width="9.14"/>
+    <col customWidth="1" min="12" max="12" width="8.71"/>
+    <col customWidth="1" min="13" max="13" width="11.14"/>
+    <col customWidth="1" min="14" max="14" width="6.29"/>
+    <col customWidth="1" min="15" max="15" width="5.0"/>
+    <col customWidth="1" min="16" max="16" width="5.14"/>
+    <col customWidth="1" min="17" max="17" width="5.71"/>
+    <col customWidth="1" min="18" max="18" width="10.43"/>
     <col customWidth="1" min="19" max="22" width="8.71"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" ht="8.25" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1328,9 +1343,23 @@
       <c r="C2" s="3"/>
       <c r="D2" s="4"/>
       <c r="E2" s="5"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="7"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="9"/>
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
@@ -1340,16 +1369,24 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" ht="15.0" customHeight="1">
+    <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="1"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="11"/>
-      <c r="P3" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="13"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="12"/>
       <c r="R3" s="14"/>
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
@@ -1362,23 +1399,23 @@
     </row>
     <row r="4" ht="3.0" customHeight="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15"/>
       <c r="S4" s="1"/>
       <c r="T4" s="1"/>
       <c r="U4" s="1"/>
@@ -1390,29 +1427,29 @@
     </row>
     <row r="5" ht="25.5" customHeight="1">
       <c r="A5" s="1"/>
-      <c r="B5" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="16" t="s">
+      <c r="B5" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="17"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="19" t="s">
+      <c r="C5" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
-      <c r="O5" s="18"/>
-      <c r="P5" s="20"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="4"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="9"/>
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
       <c r="U5" s="1"/>
@@ -1426,24 +1463,24 @@
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="24"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="14"/>
-      <c r="P6" s="25"/>
-      <c r="R6" s="26"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="24"/>
+      <c r="N6" s="24"/>
+      <c r="O6" s="25"/>
+      <c r="P6" s="27"/>
+      <c r="R6" s="28"/>
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
@@ -1455,30 +1492,30 @@
     </row>
     <row r="7" ht="33.75" customHeight="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="28" t="s">
-        <v>8</v>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="30" t="s">
+        <v>5</v>
       </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="14"/>
-      <c r="P7" s="25"/>
-      <c r="R7" s="26"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24"/>
+      <c r="N7" s="24"/>
+      <c r="O7" s="25"/>
+      <c r="P7" s="27"/>
+      <c r="R7" s="28"/>
       <c r="S7" s="1"/>
-      <c r="T7" s="29"/>
-      <c r="U7" s="29"/>
-      <c r="V7" s="29"/>
+      <c r="T7" s="31"/>
+      <c r="U7" s="31"/>
+      <c r="V7" s="31"/>
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
@@ -1486,36 +1523,36 @@
     </row>
     <row r="8" ht="36.0" customHeight="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" s="12"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="31" t="s">
+      <c r="J8" s="24"/>
+      <c r="K8" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="L8" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="32"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="34" t="s">
+      <c r="M8" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="J8" s="13"/>
-      <c r="K8" s="35">
-        <v>26.0</v>
-      </c>
-      <c r="L8" s="36" t="s">
-        <v>12</v>
-      </c>
-      <c r="M8" s="37" t="s">
-        <v>13</v>
-      </c>
       <c r="N8" s="38" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="O8" s="39"/>
-      <c r="P8" s="25"/>
-      <c r="R8" s="26"/>
+      <c r="P8" s="27"/>
+      <c r="R8" s="28"/>
       <c r="S8" s="1"/>
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
@@ -1527,35 +1564,37 @@
     </row>
     <row r="9" ht="31.5" customHeight="1">
       <c r="A9" s="1"/>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="12"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" s="25"/>
+      <c r="K9" s="41" t="s">
+        <v>5</v>
+      </c>
+      <c r="L9" s="13"/>
+      <c r="M9" s="42" t="s">
+        <v>14</v>
+      </c>
+      <c r="N9" s="43" t="s">
+        <v>5</v>
+      </c>
+      <c r="O9" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="32"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="41" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" s="14"/>
-      <c r="K9" s="42" t="s">
-        <v>18</v>
-      </c>
-      <c r="L9" s="33"/>
-      <c r="M9" s="43" t="s">
-        <v>19</v>
-      </c>
-      <c r="N9" s="44"/>
-      <c r="O9" s="45" t="s">
-        <v>20</v>
-      </c>
-      <c r="P9" s="46"/>
-      <c r="Q9" s="32"/>
-      <c r="R9" s="47"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="14"/>
       <c r="S9" s="1"/>
       <c r="T9" s="1"/>
       <c r="U9" s="1"/>
@@ -1567,42 +1606,44 @@
     </row>
     <row r="10" ht="33.0" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" s="40" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="25"/>
+      <c r="I10" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J10" s="25"/>
+      <c r="K10" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="L10" s="47" t="s">
+        <v>5</v>
+      </c>
+      <c r="M10" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="N10" s="48" t="s">
+        <v>5</v>
+      </c>
+      <c r="O10" s="49" t="s">
+        <v>20</v>
+      </c>
+      <c r="P10" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="48" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" s="41" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" s="14"/>
-      <c r="I10" s="28" t="s">
-        <v>24</v>
-      </c>
-      <c r="J10" s="14"/>
-      <c r="K10" s="49" t="s">
-        <v>25</v>
-      </c>
-      <c r="L10" s="50" t="s">
-        <v>26</v>
-      </c>
-      <c r="M10" s="43" t="s">
-        <v>27</v>
-      </c>
-      <c r="N10" s="51"/>
-      <c r="O10" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="P10" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q10" s="14"/>
-      <c r="R10" s="53" t="s">
-        <v>30</v>
+      <c r="Q10" s="25"/>
+      <c r="R10" s="50" t="s">
+        <v>5</v>
       </c>
       <c r="S10" s="1"/>
       <c r="T10" s="1"/>
@@ -1615,33 +1656,33 @@
     </row>
     <row r="11" ht="30.75" customHeight="1">
       <c r="A11" s="1"/>
-      <c r="B11" s="54" t="s">
-        <v>31</v>
+      <c r="B11" s="51" t="s">
+        <v>22</v>
       </c>
-      <c r="C11" s="55"/>
-      <c r="D11" s="55"/>
+      <c r="C11" s="52"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="39"/>
-      <c r="F11" s="41" t="s">
-        <v>32</v>
+      <c r="F11" s="40" t="s">
+        <v>23</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="49" t="s">
-        <v>33</v>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="25"/>
+      <c r="K11" s="46" t="s">
+        <v>24</v>
       </c>
-      <c r="L11" s="41" t="s">
-        <v>34</v>
+      <c r="L11" s="40" t="s">
+        <v>25</v>
       </c>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="14"/>
-      <c r="Q11" s="41" t="s">
-        <v>35</v>
+      <c r="M11" s="24"/>
+      <c r="N11" s="24"/>
+      <c r="O11" s="24"/>
+      <c r="P11" s="25"/>
+      <c r="Q11" s="40" t="s">
+        <v>26</v>
       </c>
-      <c r="R11" s="56"/>
+      <c r="R11" s="53"/>
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
@@ -1653,23 +1694,37 @@
     </row>
     <row r="12" ht="33.0" customHeight="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="11"/>
-      <c r="E12" s="57"/>
-      <c r="F12" s="58"/>
-      <c r="G12" s="59"/>
-      <c r="H12" s="45" t="s">
-        <v>36</v>
+      <c r="B12" s="54"/>
+      <c r="E12" s="55"/>
+      <c r="F12" s="30" t="s">
+        <v>5</v>
       </c>
-      <c r="I12" s="58"/>
-      <c r="J12" s="59"/>
-      <c r="K12" s="50"/>
-      <c r="L12" s="28"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="13"/>
-      <c r="O12" s="13"/>
-      <c r="P12" s="14"/>
-      <c r="Q12" s="28"/>
-      <c r="R12" s="56"/>
+      <c r="G12" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="H12" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="I12" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J12" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="K12" s="47" t="s">
+        <v>5</v>
+      </c>
+      <c r="L12" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="M12" s="24"/>
+      <c r="N12" s="24"/>
+      <c r="O12" s="24"/>
+      <c r="P12" s="25"/>
+      <c r="Q12" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="R12" s="53"/>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
@@ -1681,23 +1736,37 @@
     </row>
     <row r="13" ht="32.25" customHeight="1">
       <c r="A13" s="1"/>
-      <c r="B13" s="11"/>
-      <c r="E13" s="57"/>
-      <c r="F13" s="58"/>
-      <c r="G13" s="59"/>
-      <c r="H13" s="45" t="s">
-        <v>36</v>
+      <c r="B13" s="54"/>
+      <c r="E13" s="55"/>
+      <c r="F13" s="30" t="s">
+        <v>5</v>
       </c>
-      <c r="I13" s="58"/>
-      <c r="J13" s="59"/>
-      <c r="K13" s="50"/>
-      <c r="L13" s="28"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
-      <c r="P13" s="14"/>
-      <c r="Q13" s="28"/>
-      <c r="R13" s="56"/>
+      <c r="G13" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="H13" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="I13" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J13" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="K13" s="47" t="s">
+        <v>5</v>
+      </c>
+      <c r="L13" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="M13" s="24"/>
+      <c r="N13" s="24"/>
+      <c r="O13" s="24"/>
+      <c r="P13" s="25"/>
+      <c r="Q13" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="R13" s="53"/>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
@@ -1709,23 +1778,37 @@
     </row>
     <row r="14" ht="28.5" customHeight="1">
       <c r="A14" s="1"/>
-      <c r="B14" s="11"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="58"/>
-      <c r="G14" s="59"/>
-      <c r="H14" s="45" t="s">
-        <v>36</v>
+      <c r="B14" s="54"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="30" t="s">
+        <v>5</v>
       </c>
-      <c r="I14" s="58"/>
-      <c r="J14" s="59"/>
-      <c r="K14" s="50"/>
-      <c r="L14" s="28"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="14"/>
-      <c r="Q14" s="28"/>
-      <c r="R14" s="56"/>
+      <c r="G14" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="H14" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="I14" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J14" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="K14" s="47" t="s">
+        <v>5</v>
+      </c>
+      <c r="L14" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="M14" s="24"/>
+      <c r="N14" s="24"/>
+      <c r="O14" s="24"/>
+      <c r="P14" s="25"/>
+      <c r="Q14" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="R14" s="53"/>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
@@ -1737,21 +1820,37 @@
     </row>
     <row r="15" ht="29.25" customHeight="1">
       <c r="A15" s="1"/>
-      <c r="B15" s="11"/>
-      <c r="E15" s="57"/>
-      <c r="F15" s="58"/>
-      <c r="G15" s="59"/>
-      <c r="H15" s="45"/>
-      <c r="I15" s="58"/>
-      <c r="J15" s="59"/>
-      <c r="K15" s="50"/>
-      <c r="L15" s="28"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="14"/>
-      <c r="Q15" s="28"/>
-      <c r="R15" s="56"/>
+      <c r="B15" s="54"/>
+      <c r="E15" s="55"/>
+      <c r="F15" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="H15" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="I15" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J15" s="56" t="s">
+        <v>5</v>
+      </c>
+      <c r="K15" s="47" t="s">
+        <v>5</v>
+      </c>
+      <c r="L15" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="M15" s="24"/>
+      <c r="N15" s="24"/>
+      <c r="O15" s="24"/>
+      <c r="P15" s="25"/>
+      <c r="Q15" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="R15" s="53"/>
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
@@ -1763,35 +1862,35 @@
     </row>
     <row r="16" ht="42.75" customHeight="1">
       <c r="A16" s="1"/>
-      <c r="B16" s="60" t="s">
-        <v>37</v>
+      <c r="B16" s="57" t="s">
+        <v>28</v>
       </c>
-      <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
+      <c r="C16" s="52"/>
+      <c r="D16" s="52"/>
       <c r="E16" s="39"/>
-      <c r="F16" s="61" t="s">
+      <c r="F16" s="58" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="59"/>
+      <c r="H16" s="40" t="s">
+        <v>29</v>
+      </c>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="40" t="s">
+        <v>30</v>
+      </c>
+      <c r="M16" s="25"/>
+      <c r="N16" s="40" t="s">
+        <v>31</v>
+      </c>
+      <c r="O16" s="24"/>
+      <c r="P16" s="25"/>
+      <c r="Q16" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="G16" s="62"/>
-      <c r="H16" s="41" t="s">
-        <v>38</v>
-      </c>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="41" t="s">
-        <v>39</v>
-      </c>
-      <c r="M16" s="14"/>
-      <c r="N16" s="41" t="s">
-        <v>40</v>
-      </c>
-      <c r="O16" s="13"/>
-      <c r="P16" s="14"/>
-      <c r="Q16" s="41" t="s">
-        <v>41</v>
-      </c>
-      <c r="R16" s="56"/>
+      <c r="R16" s="53"/>
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
       <c r="U16" s="1"/>
@@ -1803,21 +1902,33 @@
     </row>
     <row r="17" ht="18.0" customHeight="1">
       <c r="A17" s="1"/>
-      <c r="B17" s="11"/>
-      <c r="E17" s="57"/>
-      <c r="F17" s="58"/>
-      <c r="G17" s="63"/>
-      <c r="H17" s="64"/>
-      <c r="I17" s="55"/>
-      <c r="J17" s="55"/>
+      <c r="B17" s="54"/>
+      <c r="E17" s="55"/>
+      <c r="F17" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="G17" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="H17" s="61" t="s">
+        <v>5</v>
+      </c>
+      <c r="I17" s="52"/>
+      <c r="J17" s="52"/>
       <c r="K17" s="39"/>
-      <c r="L17" s="38"/>
+      <c r="L17" s="61" t="s">
+        <v>5</v>
+      </c>
       <c r="M17" s="39"/>
-      <c r="N17" s="38"/>
-      <c r="O17" s="55"/>
+      <c r="N17" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="O17" s="52"/>
       <c r="P17" s="39"/>
-      <c r="Q17" s="38"/>
-      <c r="R17" s="65"/>
+      <c r="Q17" s="61" t="s">
+        <v>5</v>
+      </c>
+      <c r="R17" s="63"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
       <c r="U17" s="1"/>
@@ -1829,25 +1940,25 @@
     </row>
     <row r="18" ht="23.25" customHeight="1">
       <c r="A18" s="1"/>
-      <c r="B18" s="11"/>
-      <c r="E18" s="57"/>
-      <c r="F18" s="58" t="s">
-        <v>42</v>
+      <c r="B18" s="54"/>
+      <c r="E18" s="55"/>
+      <c r="F18" s="30" t="s">
+        <v>5</v>
       </c>
-      <c r="G18" s="66" t="s">
-        <v>43</v>
+      <c r="G18" s="60" t="s">
+        <v>5</v>
       </c>
-      <c r="H18" s="32"/>
-      <c r="I18" s="32"/>
-      <c r="J18" s="32"/>
-      <c r="K18" s="33"/>
-      <c r="L18" s="46"/>
-      <c r="M18" s="33"/>
-      <c r="N18" s="46"/>
-      <c r="O18" s="32"/>
-      <c r="P18" s="33"/>
-      <c r="Q18" s="46"/>
-      <c r="R18" s="47"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="11"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="11"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="13"/>
+      <c r="Q18" s="11"/>
+      <c r="R18" s="14"/>
       <c r="S18" s="1"/>
       <c r="T18" s="1"/>
       <c r="U18" s="1"/>
@@ -1859,21 +1970,33 @@
     </row>
     <row r="19" ht="18.0" customHeight="1">
       <c r="A19" s="1"/>
-      <c r="B19" s="11"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="58"/>
-      <c r="G19" s="59"/>
-      <c r="H19" s="64"/>
-      <c r="I19" s="55"/>
-      <c r="J19" s="55"/>
+      <c r="B19" s="54"/>
+      <c r="E19" s="55"/>
+      <c r="F19" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="G19" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="H19" s="61" t="s">
+        <v>5</v>
+      </c>
+      <c r="I19" s="52"/>
+      <c r="J19" s="52"/>
       <c r="K19" s="39"/>
-      <c r="L19" s="38"/>
+      <c r="L19" s="61" t="s">
+        <v>5</v>
+      </c>
       <c r="M19" s="39"/>
-      <c r="N19" s="38"/>
-      <c r="O19" s="55"/>
+      <c r="N19" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="O19" s="52"/>
       <c r="P19" s="39"/>
-      <c r="Q19" s="38"/>
-      <c r="R19" s="65"/>
+      <c r="Q19" s="61" t="s">
+        <v>5</v>
+      </c>
+      <c r="R19" s="63"/>
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
       <c r="U19" s="1"/>
@@ -1885,21 +2008,25 @@
     </row>
     <row r="20" ht="21.0" customHeight="1">
       <c r="A20" s="1"/>
-      <c r="B20" s="11"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="58"/>
-      <c r="G20" s="59"/>
-      <c r="H20" s="32"/>
-      <c r="I20" s="32"/>
-      <c r="J20" s="32"/>
-      <c r="K20" s="33"/>
-      <c r="L20" s="46"/>
-      <c r="M20" s="33"/>
-      <c r="N20" s="46"/>
-      <c r="O20" s="32"/>
-      <c r="P20" s="33"/>
-      <c r="Q20" s="46"/>
-      <c r="R20" s="47"/>
+      <c r="B20" s="54"/>
+      <c r="E20" s="55"/>
+      <c r="F20" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="G20" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="H20" s="11"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="11"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="11"/>
+      <c r="O20" s="12"/>
+      <c r="P20" s="13"/>
+      <c r="Q20" s="11"/>
+      <c r="R20" s="14"/>
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
       <c r="U20" s="1"/>
@@ -1911,21 +2038,33 @@
     </row>
     <row r="21" ht="18.0" customHeight="1">
       <c r="A21" s="1"/>
-      <c r="B21" s="11"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="58"/>
-      <c r="G21" s="59"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="55"/>
-      <c r="J21" s="55"/>
+      <c r="B21" s="54"/>
+      <c r="E21" s="55"/>
+      <c r="F21" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="G21" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="H21" s="61" t="s">
+        <v>5</v>
+      </c>
+      <c r="I21" s="52"/>
+      <c r="J21" s="52"/>
       <c r="K21" s="39"/>
-      <c r="L21" s="38"/>
+      <c r="L21" s="61" t="s">
+        <v>5</v>
+      </c>
       <c r="M21" s="39"/>
-      <c r="N21" s="38"/>
-      <c r="O21" s="55"/>
+      <c r="N21" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="O21" s="52"/>
       <c r="P21" s="39"/>
-      <c r="Q21" s="38"/>
-      <c r="R21" s="65"/>
+      <c r="Q21" s="61" t="s">
+        <v>5</v>
+      </c>
+      <c r="R21" s="63"/>
       <c r="S21" s="1"/>
       <c r="T21" s="1"/>
       <c r="U21" s="1"/>
@@ -1937,21 +2076,25 @@
     </row>
     <row r="22" ht="21.75" customHeight="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="11"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="58"/>
-      <c r="G22" s="59"/>
-      <c r="H22" s="46"/>
-      <c r="I22" s="32"/>
-      <c r="J22" s="32"/>
-      <c r="K22" s="33"/>
-      <c r="L22" s="46"/>
-      <c r="M22" s="33"/>
-      <c r="N22" s="46"/>
-      <c r="O22" s="32"/>
-      <c r="P22" s="33"/>
-      <c r="Q22" s="46"/>
-      <c r="R22" s="47"/>
+      <c r="B22" s="54"/>
+      <c r="E22" s="55"/>
+      <c r="F22" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="G22" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="H22" s="11"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="11"/>
+      <c r="O22" s="12"/>
+      <c r="P22" s="13"/>
+      <c r="Q22" s="11"/>
+      <c r="R22" s="14"/>
       <c r="S22" s="1"/>
       <c r="T22" s="1"/>
       <c r="U22" s="1"/>
@@ -1963,21 +2106,33 @@
     </row>
     <row r="23" ht="18.0" customHeight="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="11"/>
-      <c r="E23" s="57"/>
-      <c r="F23" s="58"/>
-      <c r="G23" s="59"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="55"/>
-      <c r="J23" s="55"/>
+      <c r="B23" s="54"/>
+      <c r="E23" s="55"/>
+      <c r="F23" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="G23" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="H23" s="61" t="s">
+        <v>5</v>
+      </c>
+      <c r="I23" s="52"/>
+      <c r="J23" s="52"/>
       <c r="K23" s="39"/>
-      <c r="L23" s="38"/>
+      <c r="L23" s="61" t="s">
+        <v>5</v>
+      </c>
       <c r="M23" s="39"/>
-      <c r="N23" s="67"/>
-      <c r="O23" s="55"/>
+      <c r="N23" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="O23" s="52"/>
       <c r="P23" s="39"/>
-      <c r="Q23" s="38"/>
-      <c r="R23" s="65"/>
+      <c r="Q23" s="61" t="s">
+        <v>5</v>
+      </c>
+      <c r="R23" s="63"/>
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
       <c r="U23" s="1"/>
@@ -1989,23 +2144,27 @@
     </row>
     <row r="24" ht="21.75" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="68"/>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="58"/>
-      <c r="G24" s="59"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="32"/>
-      <c r="J24" s="32"/>
-      <c r="K24" s="33"/>
-      <c r="L24" s="46"/>
-      <c r="M24" s="33"/>
-      <c r="N24" s="46"/>
-      <c r="O24" s="32"/>
-      <c r="P24" s="33"/>
-      <c r="Q24" s="46"/>
-      <c r="R24" s="47"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="G24" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="H24" s="11"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="11"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="11"/>
+      <c r="O24" s="12"/>
+      <c r="P24" s="13"/>
+      <c r="Q24" s="11"/>
+      <c r="R24" s="14"/>
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
       <c r="U24" s="1"/>
@@ -2017,27 +2176,37 @@
     </row>
     <row r="25" ht="33.75" customHeight="1">
       <c r="A25" s="1"/>
-      <c r="B25" s="60" t="s">
-        <v>44</v>
+      <c r="B25" s="57" t="s">
+        <v>33</v>
       </c>
-      <c r="C25" s="55"/>
-      <c r="D25" s="55"/>
+      <c r="C25" s="52"/>
+      <c r="D25" s="52"/>
       <c r="E25" s="39"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="69"/>
-      <c r="J25" s="52"/>
-      <c r="K25" s="41" t="s">
-        <v>45</v>
+      <c r="F25" s="64" t="s">
+        <v>34</v>
       </c>
-      <c r="L25" s="14"/>
-      <c r="M25" s="50"/>
-      <c r="N25" s="28"/>
-      <c r="O25" s="13"/>
-      <c r="P25" s="13"/>
-      <c r="Q25" s="13"/>
-      <c r="R25" s="56"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="25"/>
+      <c r="I25" s="65" t="s">
+        <v>5</v>
+      </c>
+      <c r="J25" s="66" t="s">
+        <v>5</v>
+      </c>
+      <c r="K25" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="L25" s="25"/>
+      <c r="M25" s="47" t="s">
+        <v>5</v>
+      </c>
+      <c r="N25" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="O25" s="24"/>
+      <c r="P25" s="24"/>
+      <c r="Q25" s="24"/>
+      <c r="R25" s="53"/>
       <c r="S25" s="1"/>
       <c r="T25" s="1"/>
       <c r="U25" s="1"/>
@@ -2049,25 +2218,35 @@
     </row>
     <row r="26" ht="33.0" customHeight="1">
       <c r="A26" s="1"/>
-      <c r="B26" s="68"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="70"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="71"/>
-      <c r="J26" s="52"/>
-      <c r="K26" s="41" t="s">
-        <v>46</v>
+      <c r="B26" s="10"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="67" t="s">
+        <v>36</v>
       </c>
-      <c r="L26" s="14"/>
-      <c r="M26" s="50"/>
-      <c r="N26" s="28"/>
-      <c r="O26" s="13"/>
-      <c r="P26" s="13"/>
-      <c r="Q26" s="13"/>
-      <c r="R26" s="56"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="68" t="s">
+        <v>5</v>
+      </c>
+      <c r="J26" s="66" t="s">
+        <v>5</v>
+      </c>
+      <c r="K26" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="L26" s="25"/>
+      <c r="M26" s="47" t="s">
+        <v>5</v>
+      </c>
+      <c r="N26" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="O26" s="24"/>
+      <c r="P26" s="24"/>
+      <c r="Q26" s="24"/>
+      <c r="R26" s="53"/>
       <c r="S26" s="1"/>
       <c r="T26" s="1"/>
       <c r="U26" s="1"/>
@@ -2079,25 +2258,25 @@
     </row>
     <row r="27" ht="25.5" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="30" t="s">
-        <v>47</v>
+      <c r="B27" s="32" t="s">
+        <v>38</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
-      <c r="J27" s="13"/>
-      <c r="K27" s="13"/>
-      <c r="L27" s="13"/>
-      <c r="M27" s="13"/>
-      <c r="N27" s="13"/>
-      <c r="O27" s="13"/>
-      <c r="P27" s="13"/>
-      <c r="Q27" s="13"/>
-      <c r="R27" s="56"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
+      <c r="L27" s="24"/>
+      <c r="M27" s="24"/>
+      <c r="N27" s="24"/>
+      <c r="O27" s="24"/>
+      <c r="P27" s="24"/>
+      <c r="Q27" s="24"/>
+      <c r="R27" s="53"/>
       <c r="S27" s="1"/>
       <c r="T27" s="1"/>
       <c r="U27" s="1"/>
@@ -2109,31 +2288,31 @@
     </row>
     <row r="28" ht="33.0" customHeight="1">
       <c r="A28" s="1"/>
-      <c r="B28" s="30" t="s">
-        <v>48</v>
+      <c r="B28" s="32" t="s">
+        <v>39</v>
       </c>
-      <c r="C28" s="14"/>
-      <c r="D28" s="41" t="s">
-        <v>2</v>
+      <c r="C28" s="25"/>
+      <c r="D28" s="40" t="s">
+        <v>3</v>
       </c>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="41" t="s">
-        <v>11</v>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="40" t="s">
+        <v>9</v>
       </c>
-      <c r="J28" s="14"/>
-      <c r="K28" s="41" t="s">
-        <v>49</v>
+      <c r="J28" s="25"/>
+      <c r="K28" s="40" t="s">
+        <v>40</v>
       </c>
-      <c r="L28" s="13"/>
-      <c r="M28" s="13"/>
-      <c r="N28" s="13"/>
-      <c r="O28" s="13"/>
-      <c r="P28" s="13"/>
-      <c r="Q28" s="13"/>
-      <c r="R28" s="56"/>
+      <c r="L28" s="24"/>
+      <c r="M28" s="24"/>
+      <c r="N28" s="24"/>
+      <c r="O28" s="24"/>
+      <c r="P28" s="24"/>
+      <c r="Q28" s="24"/>
+      <c r="R28" s="53"/>
       <c r="S28" s="1"/>
       <c r="T28" s="1"/>
       <c r="U28" s="1"/>
@@ -2145,23 +2324,31 @@
     </row>
     <row r="29" ht="18.75" customHeight="1">
       <c r="A29" s="1"/>
-      <c r="B29" s="72"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="14"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="13"/>
-      <c r="M29" s="13"/>
-      <c r="N29" s="13"/>
-      <c r="O29" s="13"/>
-      <c r="P29" s="13"/>
-      <c r="Q29" s="13"/>
-      <c r="R29" s="56"/>
+      <c r="B29" s="69" t="s">
+        <v>5</v>
+      </c>
+      <c r="C29" s="25"/>
+      <c r="D29" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="25"/>
+      <c r="I29" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J29" s="25"/>
+      <c r="K29" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="L29" s="24"/>
+      <c r="M29" s="24"/>
+      <c r="N29" s="24"/>
+      <c r="O29" s="24"/>
+      <c r="P29" s="24"/>
+      <c r="Q29" s="24"/>
+      <c r="R29" s="53"/>
       <c r="S29" s="1"/>
       <c r="T29" s="1"/>
       <c r="U29" s="1"/>
@@ -2173,23 +2360,31 @@
     </row>
     <row r="30" ht="17.25" customHeight="1">
       <c r="A30" s="1"/>
-      <c r="B30" s="72"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="28"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="14"/>
-      <c r="K30" s="28"/>
-      <c r="L30" s="13"/>
-      <c r="M30" s="13"/>
-      <c r="N30" s="13"/>
-      <c r="O30" s="13"/>
-      <c r="P30" s="13"/>
-      <c r="Q30" s="13"/>
-      <c r="R30" s="56"/>
+      <c r="B30" s="69" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="25"/>
+      <c r="D30" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J30" s="25"/>
+      <c r="K30" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="L30" s="24"/>
+      <c r="M30" s="24"/>
+      <c r="N30" s="24"/>
+      <c r="O30" s="24"/>
+      <c r="P30" s="24"/>
+      <c r="Q30" s="24"/>
+      <c r="R30" s="53"/>
       <c r="S30" s="1"/>
       <c r="T30" s="1"/>
       <c r="U30" s="1"/>
@@ -2201,23 +2396,31 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="1"/>
-      <c r="B31" s="72"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="28"/>
-      <c r="L31" s="13"/>
-      <c r="M31" s="13"/>
-      <c r="N31" s="13"/>
-      <c r="O31" s="13"/>
-      <c r="P31" s="13"/>
-      <c r="Q31" s="13"/>
-      <c r="R31" s="56"/>
+      <c r="B31" s="69" t="s">
+        <v>5</v>
+      </c>
+      <c r="C31" s="25"/>
+      <c r="D31" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="25"/>
+      <c r="I31" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J31" s="25"/>
+      <c r="K31" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="L31" s="24"/>
+      <c r="M31" s="24"/>
+      <c r="N31" s="24"/>
+      <c r="O31" s="24"/>
+      <c r="P31" s="24"/>
+      <c r="Q31" s="24"/>
+      <c r="R31" s="53"/>
       <c r="S31" s="1"/>
       <c r="T31" s="1"/>
       <c r="U31" s="1"/>
@@ -2229,23 +2432,31 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="1"/>
-      <c r="B32" s="72"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="14"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="13"/>
-      <c r="M32" s="13"/>
-      <c r="N32" s="13"/>
-      <c r="O32" s="13"/>
-      <c r="P32" s="13"/>
-      <c r="Q32" s="13"/>
-      <c r="R32" s="56"/>
+      <c r="B32" s="69" t="s">
+        <v>5</v>
+      </c>
+      <c r="C32" s="25"/>
+      <c r="D32" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="25"/>
+      <c r="I32" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J32" s="25"/>
+      <c r="K32" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="L32" s="24"/>
+      <c r="M32" s="24"/>
+      <c r="N32" s="24"/>
+      <c r="O32" s="24"/>
+      <c r="P32" s="24"/>
+      <c r="Q32" s="24"/>
+      <c r="R32" s="53"/>
       <c r="S32" s="1"/>
       <c r="T32" s="1"/>
       <c r="U32" s="1"/>
@@ -2257,23 +2468,31 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="1"/>
-      <c r="B33" s="73"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="74"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="74"/>
-      <c r="J33" s="14"/>
-      <c r="K33" s="74"/>
-      <c r="L33" s="13"/>
-      <c r="M33" s="13"/>
-      <c r="N33" s="13"/>
-      <c r="O33" s="13"/>
-      <c r="P33" s="13"/>
-      <c r="Q33" s="13"/>
-      <c r="R33" s="56"/>
+      <c r="B33" s="69" t="s">
+        <v>5</v>
+      </c>
+      <c r="C33" s="25"/>
+      <c r="D33" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J33" s="25"/>
+      <c r="K33" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="L33" s="24"/>
+      <c r="M33" s="24"/>
+      <c r="N33" s="24"/>
+      <c r="O33" s="24"/>
+      <c r="P33" s="24"/>
+      <c r="Q33" s="24"/>
+      <c r="R33" s="53"/>
       <c r="S33" s="1"/>
       <c r="T33" s="1"/>
       <c r="U33" s="1"/>
@@ -2285,25 +2504,33 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="1"/>
-      <c r="B34" s="73"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="74"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="74"/>
-      <c r="J34" s="14"/>
-      <c r="K34" s="74"/>
-      <c r="L34" s="13"/>
-      <c r="M34" s="13"/>
-      <c r="N34" s="13"/>
-      <c r="O34" s="13"/>
-      <c r="P34" s="13"/>
-      <c r="Q34" s="13"/>
-      <c r="R34" s="56"/>
+      <c r="B34" s="69" t="s">
+        <v>5</v>
+      </c>
+      <c r="C34" s="25"/>
+      <c r="D34" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="25"/>
+      <c r="I34" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J34" s="25"/>
+      <c r="K34" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="L34" s="24"/>
+      <c r="M34" s="24"/>
+      <c r="N34" s="24"/>
+      <c r="O34" s="24"/>
+      <c r="P34" s="24"/>
+      <c r="Q34" s="24"/>
+      <c r="R34" s="53"/>
       <c r="S34" s="1"/>
-      <c r="T34" s="1"/>
+      <c r="T34" s="70"/>
       <c r="U34" s="1"/>
       <c r="V34" s="1"/>
       <c r="W34" s="1"/>
@@ -2313,23 +2540,31 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="1"/>
-      <c r="B35" s="73"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="74"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="74"/>
-      <c r="J35" s="14"/>
-      <c r="K35" s="74"/>
-      <c r="L35" s="13"/>
-      <c r="M35" s="13"/>
-      <c r="N35" s="13"/>
-      <c r="O35" s="13"/>
-      <c r="P35" s="13"/>
-      <c r="Q35" s="13"/>
-      <c r="R35" s="56"/>
+      <c r="B35" s="69" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35" s="25"/>
+      <c r="D35" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="25"/>
+      <c r="I35" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="J35" s="25"/>
+      <c r="K35" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="L35" s="24"/>
+      <c r="M35" s="24"/>
+      <c r="N35" s="24"/>
+      <c r="O35" s="24"/>
+      <c r="P35" s="24"/>
+      <c r="Q35" s="24"/>
+      <c r="R35" s="53"/>
       <c r="S35" s="1"/>
       <c r="T35" s="1"/>
       <c r="U35" s="1"/>
@@ -2339,33 +2574,37 @@
       <c r="Y35" s="1"/>
       <c r="Z35" s="1"/>
     </row>
-    <row r="36" ht="18.0" customHeight="1">
+    <row r="36" ht="20.25" customHeight="1">
       <c r="A36" s="1"/>
-      <c r="B36" s="75" t="s">
-        <v>50</v>
+      <c r="B36" s="71" t="s">
+        <v>41</v>
       </c>
-      <c r="C36" s="76"/>
-      <c r="D36" s="76"/>
-      <c r="E36" s="62"/>
-      <c r="F36" s="77" t="s">
-        <v>51</v>
+      <c r="C36" s="72"/>
+      <c r="D36" s="72"/>
+      <c r="E36" s="59"/>
+      <c r="F36" s="73" t="s">
+        <v>42</v>
       </c>
-      <c r="G36" s="78"/>
-      <c r="H36" s="55"/>
-      <c r="I36" s="55"/>
+      <c r="G36" s="74" t="s">
+        <v>5</v>
+      </c>
+      <c r="H36" s="52"/>
+      <c r="I36" s="52"/>
       <c r="J36" s="39"/>
-      <c r="K36" s="79"/>
+      <c r="K36" s="75" t="s">
+        <v>5</v>
+      </c>
       <c r="L36" s="39"/>
-      <c r="M36" s="80" t="s">
-        <v>52</v>
+      <c r="M36" s="76" t="s">
+        <v>43</v>
       </c>
-      <c r="N36" s="81" t="s">
-        <v>16</v>
+      <c r="N36" s="77" t="s">
+        <v>5</v>
       </c>
-      <c r="O36" s="55"/>
-      <c r="P36" s="55"/>
-      <c r="Q36" s="55"/>
-      <c r="R36" s="65"/>
+      <c r="O36" s="52"/>
+      <c r="P36" s="52"/>
+      <c r="Q36" s="52"/>
+      <c r="R36" s="63"/>
       <c r="S36" s="1"/>
       <c r="T36" s="1"/>
       <c r="U36" s="1"/>
@@ -2377,25 +2616,29 @@
     </row>
     <row r="37" ht="18.0" customHeight="1">
       <c r="A37" s="1"/>
-      <c r="B37" s="82" t="s">
-        <v>53</v>
+      <c r="B37" s="78" t="s">
+        <v>44</v>
       </c>
-      <c r="C37" s="83"/>
-      <c r="D37" s="83"/>
-      <c r="E37" s="84"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
-      <c r="I37" s="32"/>
-      <c r="J37" s="33"/>
-      <c r="K37" s="46"/>
-      <c r="L37" s="33"/>
-      <c r="M37" s="46"/>
-      <c r="N37" s="32"/>
-      <c r="O37" s="32"/>
-      <c r="P37" s="32"/>
-      <c r="Q37" s="32"/>
-      <c r="R37" s="47"/>
+      <c r="C37" s="79"/>
+      <c r="D37" s="79"/>
+      <c r="E37" s="80"/>
+      <c r="F37" s="81" t="s">
+        <v>45</v>
+      </c>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="12"/>
+      <c r="J37" s="13"/>
+      <c r="K37" s="11"/>
+      <c r="L37" s="13"/>
+      <c r="M37" s="82" t="s">
+        <v>46</v>
+      </c>
+      <c r="N37" s="12"/>
+      <c r="O37" s="12"/>
+      <c r="P37" s="12"/>
+      <c r="Q37" s="12"/>
+      <c r="R37" s="14"/>
       <c r="S37" s="1"/>
       <c r="T37" s="1"/>
       <c r="U37" s="1"/>
@@ -2407,25 +2650,27 @@
     </row>
     <row r="38" ht="18.0" customHeight="1">
       <c r="A38" s="1"/>
-      <c r="B38" s="75" t="s">
-        <v>54</v>
+      <c r="B38" s="83" t="s">
+        <v>47</v>
       </c>
-      <c r="C38" s="76"/>
-      <c r="D38" s="76"/>
-      <c r="E38" s="62"/>
-      <c r="F38" s="85"/>
-      <c r="G38" s="55"/>
-      <c r="H38" s="55"/>
-      <c r="I38" s="55"/>
-      <c r="J38" s="55"/>
-      <c r="K38" s="55"/>
-      <c r="L38" s="55"/>
-      <c r="M38" s="55"/>
-      <c r="N38" s="55"/>
-      <c r="O38" s="55"/>
-      <c r="P38" s="55"/>
-      <c r="Q38" s="55"/>
-      <c r="R38" s="65"/>
+      <c r="C38" s="72"/>
+      <c r="D38" s="72"/>
+      <c r="E38" s="59"/>
+      <c r="F38" s="84" t="s">
+        <v>5</v>
+      </c>
+      <c r="G38" s="52"/>
+      <c r="H38" s="52"/>
+      <c r="I38" s="52"/>
+      <c r="J38" s="52"/>
+      <c r="K38" s="52"/>
+      <c r="L38" s="52"/>
+      <c r="M38" s="52"/>
+      <c r="N38" s="52"/>
+      <c r="O38" s="52"/>
+      <c r="P38" s="52"/>
+      <c r="Q38" s="52"/>
+      <c r="R38" s="63"/>
       <c r="S38" s="1"/>
       <c r="T38" s="1"/>
       <c r="U38" s="1"/>
@@ -2437,25 +2682,14 @@
     </row>
     <row r="39" ht="18.0" customHeight="1">
       <c r="A39" s="1"/>
-      <c r="B39" s="82" t="s">
-        <v>55</v>
+      <c r="B39" s="85" t="s">
+        <v>48</v>
       </c>
-      <c r="C39" s="83"/>
-      <c r="D39" s="83"/>
-      <c r="E39" s="84"/>
-      <c r="F39" s="86"/>
-      <c r="G39" s="32"/>
-      <c r="H39" s="32"/>
-      <c r="I39" s="32"/>
-      <c r="J39" s="32"/>
-      <c r="K39" s="32"/>
-      <c r="L39" s="32"/>
-      <c r="M39" s="32"/>
-      <c r="N39" s="32"/>
-      <c r="O39" s="32"/>
-      <c r="P39" s="32"/>
-      <c r="Q39" s="32"/>
-      <c r="R39" s="47"/>
+      <c r="C39" s="79"/>
+      <c r="D39" s="79"/>
+      <c r="E39" s="80"/>
+      <c r="F39" s="27"/>
+      <c r="R39" s="28"/>
       <c r="S39" s="1"/>
       <c r="T39" s="1"/>
       <c r="U39" s="1"/>
@@ -2467,27 +2701,31 @@
     </row>
     <row r="40" ht="45.75" customHeight="1">
       <c r="A40" s="1"/>
-      <c r="B40" s="30" t="s">
-        <v>56</v>
+      <c r="B40" s="32" t="s">
+        <v>49</v>
       </c>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
-      <c r="J40" s="14"/>
-      <c r="K40" s="41" t="s">
-        <v>57</v>
+      <c r="C40" s="24"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="25"/>
+      <c r="F40" s="30" t="s">
+        <v>5</v>
       </c>
-      <c r="L40" s="14"/>
-      <c r="M40" s="28"/>
-      <c r="N40" s="13"/>
-      <c r="O40" s="13"/>
-      <c r="P40" s="13"/>
-      <c r="Q40" s="13"/>
-      <c r="R40" s="56"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="24"/>
+      <c r="I40" s="24"/>
+      <c r="J40" s="25"/>
+      <c r="K40" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="L40" s="25"/>
+      <c r="M40" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="N40" s="24"/>
+      <c r="O40" s="24"/>
+      <c r="P40" s="24"/>
+      <c r="Q40" s="24"/>
+      <c r="R40" s="53"/>
       <c r="S40" s="1"/>
       <c r="T40" s="1"/>
       <c r="U40" s="1"/>
@@ -2499,27 +2737,31 @@
     </row>
     <row r="41" ht="45.75" customHeight="1">
       <c r="A41" s="1"/>
-      <c r="B41" s="30" t="s">
-        <v>58</v>
+      <c r="B41" s="86" t="s">
+        <v>51</v>
       </c>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="28"/>
-      <c r="G41" s="13"/>
-      <c r="H41" s="13"/>
-      <c r="I41" s="13"/>
-      <c r="J41" s="14"/>
-      <c r="K41" s="41" t="s">
-        <v>59</v>
+      <c r="C41" s="52"/>
+      <c r="D41" s="52"/>
+      <c r="E41" s="39"/>
+      <c r="F41" s="38" t="s">
+        <v>5</v>
       </c>
-      <c r="L41" s="14"/>
-      <c r="M41" s="28"/>
-      <c r="N41" s="13"/>
-      <c r="O41" s="13"/>
-      <c r="P41" s="13"/>
-      <c r="Q41" s="13"/>
-      <c r="R41" s="56"/>
+      <c r="G41" s="52"/>
+      <c r="H41" s="52"/>
+      <c r="I41" s="52"/>
+      <c r="J41" s="39"/>
+      <c r="K41" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="L41" s="25"/>
+      <c r="M41" s="30" t="s">
+        <v>5</v>
+      </c>
+      <c r="N41" s="24"/>
+      <c r="O41" s="24"/>
+      <c r="P41" s="24"/>
+      <c r="Q41" s="24"/>
+      <c r="R41" s="53"/>
       <c r="S41" s="1"/>
       <c r="T41" s="1"/>
       <c r="U41" s="1"/>
@@ -2529,21 +2771,37 @@
       <c r="Y41" s="1"/>
       <c r="Z41" s="1"/>
     </row>
-    <row r="42" ht="18.0" customHeight="1">
+    <row r="42" ht="23.25" customHeight="1">
       <c r="A42" s="1"/>
       <c r="B42" s="87" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
-      <c r="C42" s="88"/>
-      <c r="D42" s="88"/>
-      <c r="E42" s="88"/>
-      <c r="F42" s="88"/>
-      <c r="G42" s="88"/>
-      <c r="H42" s="88"/>
-      <c r="I42" s="88"/>
-      <c r="J42" s="89"/>
-      <c r="K42" s="90"/>
-      <c r="R42" s="26"/>
+      <c r="C42" s="52"/>
+      <c r="D42" s="52"/>
+      <c r="E42" s="39"/>
+      <c r="F42" s="88" t="s">
+        <v>5</v>
+      </c>
+      <c r="G42" s="52"/>
+      <c r="H42" s="52"/>
+      <c r="I42" s="52"/>
+      <c r="J42" s="39"/>
+      <c r="K42" s="89" t="s">
+        <v>54</v>
+      </c>
+      <c r="L42" s="55"/>
+      <c r="M42" s="90" t="s">
+        <v>5</v>
+      </c>
+      <c r="N42" s="90" t="s">
+        <v>5</v>
+      </c>
+      <c r="P42" s="90" t="s">
+        <v>5</v>
+      </c>
+      <c r="R42" s="91" t="s">
+        <v>5</v>
+      </c>
       <c r="S42" s="1"/>
       <c r="T42" s="1"/>
       <c r="U42" s="1"/>
@@ -2553,27 +2811,29 @@
       <c r="Y42" s="1"/>
       <c r="Z42" s="1"/>
     </row>
-    <row r="43" ht="18.0" customHeight="1">
+    <row r="43" ht="24.0" customHeight="1">
       <c r="A43" s="1"/>
-      <c r="B43" s="91" t="s">
-        <v>61</v>
+      <c r="B43" s="92" t="s">
+        <v>55</v>
       </c>
-      <c r="C43" s="92"/>
-      <c r="D43" s="92"/>
-      <c r="E43" s="92"/>
-      <c r="F43" s="92"/>
-      <c r="G43" s="92"/>
-      <c r="H43" s="92"/>
-      <c r="I43" s="92"/>
-      <c r="J43" s="93"/>
-      <c r="K43" s="94"/>
-      <c r="L43" s="9"/>
-      <c r="M43" s="9"/>
-      <c r="N43" s="9"/>
-      <c r="O43" s="9"/>
-      <c r="P43" s="9"/>
-      <c r="Q43" s="9"/>
-      <c r="R43" s="10"/>
+      <c r="C43" s="93"/>
+      <c r="D43" s="93"/>
+      <c r="E43" s="94"/>
+      <c r="F43" s="93"/>
+      <c r="G43" s="93"/>
+      <c r="H43" s="93"/>
+      <c r="I43" s="93"/>
+      <c r="J43" s="94"/>
+      <c r="K43" s="95" t="s">
+        <v>56</v>
+      </c>
+      <c r="L43" s="94"/>
+      <c r="M43" s="93"/>
+      <c r="N43" s="93"/>
+      <c r="O43" s="93"/>
+      <c r="P43" s="93"/>
+      <c r="Q43" s="93"/>
+      <c r="R43" s="96"/>
       <c r="S43" s="1"/>
       <c r="T43" s="1"/>
       <c r="U43" s="1"/>
@@ -26352,28 +26612,7 @@
       <c r="V1000" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="120">
-    <mergeCell ref="N17:P18"/>
-    <mergeCell ref="Q17:R18"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="N16:P16"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="H17:K18"/>
-    <mergeCell ref="L17:M18"/>
-    <mergeCell ref="H21:K22"/>
-    <mergeCell ref="H23:K24"/>
-    <mergeCell ref="L23:M24"/>
-    <mergeCell ref="N23:P24"/>
-    <mergeCell ref="Q23:R24"/>
-    <mergeCell ref="H19:K20"/>
-    <mergeCell ref="L19:M20"/>
-    <mergeCell ref="N19:P20"/>
-    <mergeCell ref="Q19:R20"/>
-    <mergeCell ref="L21:M22"/>
-    <mergeCell ref="N21:P22"/>
-    <mergeCell ref="Q21:R22"/>
+  <mergeCells count="125">
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="C6:E6"/>
     <mergeCell ref="B5:B6"/>
@@ -26383,6 +26622,39 @@
     <mergeCell ref="B25:E26"/>
     <mergeCell ref="F25:H25"/>
     <mergeCell ref="F26:H26"/>
+    <mergeCell ref="N19:P20"/>
+    <mergeCell ref="N21:P22"/>
+    <mergeCell ref="H17:K18"/>
+    <mergeCell ref="H19:K20"/>
+    <mergeCell ref="H21:K22"/>
+    <mergeCell ref="L17:M18"/>
+    <mergeCell ref="L19:M20"/>
+    <mergeCell ref="N17:P18"/>
+    <mergeCell ref="Q17:R18"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="N25:R25"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="N26:R26"/>
+    <mergeCell ref="B27:R27"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="K30:R30"/>
+    <mergeCell ref="D30:H30"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D31:H31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="K31:R31"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="K34:R34"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="K32:R32"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="K33:R33"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
     <mergeCell ref="F7:O7"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="F8:H8"/>
@@ -26393,13 +26665,65 @@
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="G10:H10"/>
     <mergeCell ref="F11:J11"/>
+    <mergeCell ref="M42:M43"/>
+    <mergeCell ref="N42:O43"/>
     <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:D3"/>
-    <mergeCell ref="E2:O3"/>
-    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="P2:R3"/>
     <mergeCell ref="F5:O5"/>
     <mergeCell ref="P5:R9"/>
     <mergeCell ref="F6:O6"/>
+    <mergeCell ref="C2:E3"/>
+    <mergeCell ref="G2:M3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="N2:O3"/>
+    <mergeCell ref="Q19:R20"/>
+    <mergeCell ref="Q21:R22"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="K35:R35"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="H23:K24"/>
+    <mergeCell ref="L23:M24"/>
+    <mergeCell ref="N23:P24"/>
+    <mergeCell ref="Q23:R24"/>
+    <mergeCell ref="L21:M22"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="K28:R28"/>
+    <mergeCell ref="D29:H29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="K29:R29"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="G36:J37"/>
+    <mergeCell ref="K36:L37"/>
+    <mergeCell ref="N36:R37"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="F38:R39"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="F40:J40"/>
+    <mergeCell ref="K40:L40"/>
+    <mergeCell ref="M40:R40"/>
+    <mergeCell ref="P42:Q43"/>
+    <mergeCell ref="R42:R43"/>
+    <mergeCell ref="K42:L42"/>
+    <mergeCell ref="K43:L43"/>
+    <mergeCell ref="B41:E41"/>
+    <mergeCell ref="F41:J41"/>
+    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="M41:R41"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="F42:J43"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="Q16:R16"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="K9:L9"/>
     <mergeCell ref="I10:J10"/>
@@ -26407,11 +26731,6 @@
     <mergeCell ref="L11:P11"/>
     <mergeCell ref="Q11:R11"/>
     <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="N25:R25"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="N26:R26"/>
-    <mergeCell ref="B27:R27"/>
     <mergeCell ref="L12:P12"/>
     <mergeCell ref="L13:P13"/>
     <mergeCell ref="Q13:R13"/>
@@ -26419,135 +26738,7 @@
     <mergeCell ref="Q14:R14"/>
     <mergeCell ref="L15:P15"/>
     <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:H28"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="K28:R28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="K29:R29"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="K31:R31"/>
-    <mergeCell ref="K32:R32"/>
-    <mergeCell ref="K33:R33"/>
-    <mergeCell ref="K34:R34"/>
-    <mergeCell ref="K35:R35"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:H30"/>
-    <mergeCell ref="K30:R30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D31:H31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="F36:F37"/>
-    <mergeCell ref="G36:J37"/>
-    <mergeCell ref="K36:L37"/>
-    <mergeCell ref="M36:M37"/>
-    <mergeCell ref="N36:R37"/>
-    <mergeCell ref="F38:R38"/>
-    <mergeCell ref="F39:R39"/>
-    <mergeCell ref="B42:J42"/>
-    <mergeCell ref="B43:J43"/>
-    <mergeCell ref="F40:J40"/>
-    <mergeCell ref="K40:L40"/>
-    <mergeCell ref="M40:R40"/>
-    <mergeCell ref="F41:J41"/>
-    <mergeCell ref="K41:L41"/>
-    <mergeCell ref="M41:R41"/>
-    <mergeCell ref="K42:R43"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="I32:J32"/>
   </mergeCells>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8">
-      <formula1>"男            Pria,女        Wanita"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="R10 M25:M26">
-      <formula1>"有      Ada,無 Tidak"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" prompt="まだ学科名ってある？_x000a_川原に教えてください。_x000a_" sqref="Q12:Q13">
-      <formula1>"インドネシア語学科,英語学科,音楽科,外国語学科,観光学科,看護学科,機械学科,機械整備学科,漁業学科,車、バイク整備学科,経営学科,経済学科,芸能学科,経理学科,建築学科,航海学科,工業学科,コンピューター学科,裁縫学科,情報学科,助産師学科,水産学科.数学科,ソフトウェア学科,体育科,畜産学科,調理学科,デザイン学科,電気学科,電子学科,日本語学科,農学科,ビジネス学科,福祉学科,服飾科,普通科,文学科,ホテル学科,マネジメント学科,マルチメディア学科,薬学科,養殖学科,溶接学科"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F10">
-      <formula1>"A型,B型,O型,AB型,不明"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L10">
-      <formula1>"有      Ada,無 　Tidak"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="J25:J26">
-      <formula1>"週間,ヶ月,年間"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" prompt="まだ学科名ってある？_x000a_川原に教えてください。_x000a_" sqref="Q14">
-      <formula1>"看護学科,助産師学科,英語学科,外国語学科,観光学科,看護学科,機械学科,機械整備学科,漁業学科,自動車整備学科,経営学科,経済学科,芸能学科,経理学科,建築学科,航海学科,工業学科,コンピューター学科,裁縫学科,情報学科,助産師学科,水産学科.数学科,ソフトウェア学科,体育科,畜産学科,調理学科,デザイン学科,電気学科,電子学科,日本語学科,農学科,ビジネス学科,福祉学科,服飾科,普通科,文学科,ホテル学科,マネジメント学科,マルチメディア学科,薬学科,養殖学科,溶接学科,社会科学"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K9">
-      <formula1>"イスラム教　   Islam,キリスト教　  Kristen,ヒンドゥー教  Hindu,仏教　buda,カトリック    　Katrik"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L17 L19">
-      <formula1>"なし,10000円,15000円,20000円,25000円,30000円,35000円,40000円,45000円,50000円,55000円,70000円"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I10">
-      <formula1>"既婚　　　  Menikah,未婚 Single,離婚 　　 Cerai"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" prompt="まだ学科名ってある？_x000a_川原に教えてください。_x000a_" sqref="Q15">
-      <formula1>"看護学科,助産師学科,英語学科,外国語学科,観光学科,看護学科,機械学科,機械整備学科,漁業学科,自動車整備学科,経営学科,経済学科,芸能学科,経理学科,建築学科,航海学科,工業学科,コンピューター学科,裁縫学科,情報学科,助産師学科,水産学科.数学科,ソフトウェア学科,体育科,畜産学科,調理学科,デザイン学科,電気学科,電子学科,日本語学科,農学科,ビジネス学科,福祉学科,服飾科,普通科,文学科,ホテル学科,マネジメント学科,マルチメディア学科,薬学科,養殖学科,溶接学科"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B29:B35">
-      <formula1>"父 Ayah,母 Ibu,兄 Kaka cow,姉 Kakak cew,弟 Adik cowo,妹 Adik cewe,夫 Suami,妻 Istri,子供 Anak,祖父母 Kakek,叔父Paman,叔母Bibi"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L21 L23">
-      <formula1>"10000円,15000円,20000円,25000円,30000円,35000円,40000円,45000円,50000円,55000円"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I14">
-      <formula1>"1995年,1996年,1997年,1998年,1999年,2000年,2001年,2002年,2003年,2004年,2005年,2006年,2007年,2008年,2009年,2010年,2011年,2012年,2013年,2014年,2015年,2016年,2017年,2018年,2019年,2020年,2021年,2022年"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F26">
-      <formula1>"英語,韓国語,中国語,アラビア語,ドイツ語,フランス語,台湾語,ベトナム語,タイ語,スペイン語"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G12:G15 J12:J15 G17:G24">
-      <formula1>"1月,2月,3月,4月,5月,6月,7月,8月,9月,10月,11月,12月"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="K14">
-      <formula1>"普通高校　SMA,職業高校　SMK,単位高校　PaketC"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K36">
-      <formula1>"ちち,はは,あに,おとうと,あね,いもうと,おっと,つま,おじ,おば"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K15">
-      <formula1>"4年制大学D4・S1,3年制大学D3"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I25">
-      <formula1>"1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="Q17 Q19 Q21 Q23">
-      <formula1>"正社員     Karyawan tetap,契約社員 Karyawan kontrak,アルバイト           Part time,インターンシップ Magang,親の手伝い       Bantu orangtua,親戚の手伝い       Bantu Saudara,その他Lainnya"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F25">
-      <formula1>"日本語学習期間"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I12:I13 F12:F15 I15 F17:F24">
-      <formula1>"1991年,1992年,1993年,1994年,1995年,1996年,1997年,1998年,1999年,2000年,2001年,2002年,2003年,2004年,2005年,2006年,2007年,2008年,2009年,2010年,2011年,2012年,2013年,2014年,2015年,2016年,2017年,2018年,2019年,2020年"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I26">
-      <formula1>"初級,中級,上級"</formula1>
-    </dataValidation>
-  </dataValidations>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins bottom="0.5511811023622047" footer="0.0" header="0.0" left="0.7086614173228347" right="0.7086614173228347" top="0.7480314960629921"/>
   <pageSetup paperSize="9" scale="85" orientation="portrait"/>

</xml_diff>